<commit_message>
Ajout de quelques images du montage
</commit_message>
<xml_diff>
--- a/Docs/Retour d'expérience/Retour d'expérience.xlsx
+++ b/Docs/Retour d'expérience/Retour d'expérience.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Cours\Lowtech\WINS 2026\Four solaire\Docs\Retour d'expérience\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7127B0FE-A600-49FD-B9EA-3E90E4B176D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E63385BC-0374-4729-9497-DE3797859995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32340" yWindow="1545" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="37">
   <si>
     <t>Retour d'expérience sur la fabrication, le montage et l'utilisation  du four</t>
   </si>
@@ -83,6 +83,63 @@
   </si>
   <si>
     <t>Augmenter le jeu des trous avec une lime ronde / forêt plus grand (le faire parois assemblée).</t>
+  </si>
+  <si>
+    <t>Tringles</t>
+  </si>
+  <si>
+    <t>Cadre déflecteur</t>
+  </si>
+  <si>
+    <t>Les tringles utilisées Ø2,5 ne sont pas très rigides avec la longueur voulue</t>
+  </si>
+  <si>
+    <t>Raccourcir les tringles ou augmenter le Ø</t>
+  </si>
+  <si>
+    <t>Déflecteur bas</t>
+  </si>
+  <si>
+    <t>Le déflecteur ne peut pas être réglé en position actuellement.</t>
+  </si>
+  <si>
+    <t>Parois (toutes)</t>
+  </si>
+  <si>
+    <t>Boite</t>
+  </si>
+  <si>
+    <t>Les parois intérieures sont couvertes avec du papier aluminium alimentaire et c'est très fragile</t>
+  </si>
+  <si>
+    <t>Remplacer le papier alu par des panneau d'épaisseur 0.8 mm</t>
+  </si>
+  <si>
+    <t>Alternative possible</t>
+  </si>
+  <si>
+    <t>Utiliser de l'inox</t>
+  </si>
+  <si>
+    <t>Utiliser un fil nylon attaché au cadre derière</t>
+  </si>
+  <si>
+    <t>Miroirs</t>
+  </si>
+  <si>
+    <t>Déflecteurs</t>
+  </si>
+  <si>
+    <t>Les miroirs risquent de se rayer lorsqu'ils sont repliés.</t>
+  </si>
+  <si>
+    <t>Ajouter un tissus fin entre le bois et les mirois</t>
+  </si>
+  <si>
+    <t>Utiliser les tampons de chaises sur les miroirs</t>
+  </si>
+  <si>
+    <t>Changer le mécanisme de réglage</t>
   </si>
 </sst>
 </file>
@@ -139,10 +196,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -425,39 +482,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="15.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="39" style="1" customWidth="1"/>
     <col min="4" max="4" width="41.42578125" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="5" width="21.7109375" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-    </row>
-    <row r="2" spans="1:4" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+    </row>
+    <row r="2" spans="1:5" s="2" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="E2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -471,7 +532,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -485,7 +546,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -499,7 +560,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -511,6 +572,71 @@
       </c>
       <c r="D6" s="1" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modification conf et ajout photo
</commit_message>
<xml_diff>
--- a/Docs/Retour d'expérience/Retour d'expérience.xlsx
+++ b/Docs/Retour d'expérience/Retour d'expérience.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Cours\Lowtech\WINS 2026\Four solaire\Docs\Retour d'expérience\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E63385BC-0374-4729-9497-DE3797859995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F01215-CEBF-4F5B-A5C6-D44328E43FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32340" yWindow="1545" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Ajout cale de réglage au fichiers de découpe
</commit_message>
<xml_diff>
--- a/Docs/Retour d'expérience/Retour d'expérience.xlsx
+++ b/Docs/Retour d'expérience/Retour d'expérience.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Cours\Lowtech\WINS 2026\Four solaire\Docs\Retour d'expérience\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F01215-CEBF-4F5B-A5C6-D44328E43FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4520DCF-4D1A-4B6A-B00A-094814132A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
   <si>
     <t>Retour d'expérience sur la fabrication, le montage et l'utilisation  du four</t>
   </si>
@@ -73,9 +73,6 @@
     <t>La charnière ne peut pas être vissée au cadre car les épaisseurs des panneaux est trop grande</t>
   </si>
   <si>
-    <t>Changer le type de charnière pour des plus grandes.</t>
-  </si>
-  <si>
     <t>Parois latérale</t>
   </si>
   <si>
@@ -133,13 +130,31 @@
     <t>Les miroirs risquent de se rayer lorsqu'ils sont repliés.</t>
   </si>
   <si>
-    <t>Ajouter un tissus fin entre le bois et les mirois</t>
-  </si>
-  <si>
-    <t>Utiliser les tampons de chaises sur les miroirs</t>
-  </si>
-  <si>
     <t>Changer le mécanisme de réglage</t>
+  </si>
+  <si>
+    <t>Utiliser les tampons de chaises sur l'arrière des miroirs</t>
+  </si>
+  <si>
+    <t>Ajouter un tissus fin entre le bois et les mirois et sur le cadre</t>
+  </si>
+  <si>
+    <t>Changer le type de charnière pour des plus grandes (largeur environ 50mm)</t>
+  </si>
+  <si>
+    <t>Le four posé au sol est très bas. Pas bon pour le dos et l'utilisation générale</t>
+  </si>
+  <si>
+    <t>Poser le four en hauteur, sur une table ou un tabouret.</t>
+  </si>
+  <si>
+    <t>Faire un chariot sur mesure pour le déplacer en utilisant un cageot à pommes pour le surélever.</t>
+  </si>
+  <si>
+    <t>Toutes</t>
+  </si>
+  <si>
+    <t>Four entier</t>
   </si>
 </sst>
 </file>
@@ -482,14 +497,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="15.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="39" style="1" customWidth="1"/>
-    <col min="4" max="4" width="41.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="21.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="81.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="66.140625" style="1" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
@@ -515,10 +530,10 @@
         <v>4</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -557,86 +572,106 @@
         <v>13</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="E7" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="D8" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="E9" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="D10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>35</v>
+    </row>
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Premiers essais sous le soleil
</commit_message>
<xml_diff>
--- a/Docs/Retour d'expérience/Retour d'expérience.xlsx
+++ b/Docs/Retour d'expérience/Retour d'expérience.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Cours\Lowtech\WINS 2026\Four solaire\Docs\Retour d'expérience\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4520DCF-4D1A-4B6A-B00A-094814132A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3ACB41D-EE0A-441C-A58A-672D047B11B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Problèmes_Solutions" sheetId="1" r:id="rId1"/>
+    <sheet name="Mesures températures" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="62">
   <si>
     <t>Retour d'expérience sur la fabrication, le montage et l'utilisation  du four</t>
   </si>
@@ -155,6 +156,66 @@
   </si>
   <si>
     <t>Four entier</t>
+  </si>
+  <si>
+    <t>Tôles acier</t>
+  </si>
+  <si>
+    <t>La peinture noir n'adhère pas bien à la tôle.</t>
+  </si>
+  <si>
+    <t>Mieux préparer la tôle avec un bon dégraissage, voir même un léger ponçage des surface pour mieux faire accrocher la peinture</t>
+  </si>
+  <si>
+    <t>Brunissage avec produit adapté (vérifier la compatibilité alimentaire avant)</t>
+  </si>
+  <si>
+    <t>Heure de début</t>
+  </si>
+  <si>
+    <t>Heure de fin</t>
+  </si>
+  <si>
+    <t>Météo du moment</t>
+  </si>
+  <si>
+    <t>Orientation du four</t>
+  </si>
+  <si>
+    <t>Type Thermocouple</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Beau</t>
+  </si>
+  <si>
+    <t>Sud-Ouest</t>
+  </si>
+  <si>
+    <t>Angles déflecteurs (H/B)</t>
+  </si>
+  <si>
+    <t>Température extérieure [°C]</t>
+  </si>
+  <si>
+    <t>Température initiale du four [°C]</t>
+  </si>
+  <si>
+    <t>Température finale tôle/air [°C/°C]</t>
+  </si>
+  <si>
+    <t>147,7/116,6</t>
+  </si>
+  <si>
+    <t>3xT + 1xN</t>
+  </si>
+  <si>
+    <t>Remarques</t>
+  </si>
+  <si>
+    <t>La barre symbolique des 100°C a été franchie</t>
   </si>
 </sst>
 </file>
@@ -194,7 +255,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -202,17 +263,53 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -497,7 +594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" style="1" customWidth="1"/>
@@ -509,12 +606,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -672,6 +769,23 @@
       </c>
       <c r="E11" s="1" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -681,4 +795,453 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F197876-68D4-4EAB-A7AF-00772F3B6590}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:K29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.28515625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="22.5703125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" style="4" customWidth="1"/>
+    <col min="7" max="7" width="24.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.5703125" style="4" customWidth="1"/>
+    <col min="11" max="11" width="41" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.42578125" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>46253</v>
+      </c>
+      <c r="B2" s="8">
+        <v>0.44791666666666669</v>
+      </c>
+      <c r="C2" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="D2" s="3">
+        <v>27.4</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="9">
+        <v>46253</v>
+      </c>
+      <c r="H2" s="3">
+        <v>27.4</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+    </row>
+    <row r="12" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+    </row>
+    <row r="15" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+    </row>
+    <row r="16" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+    </row>
+    <row r="17" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+    </row>
+    <row r="18" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+    </row>
+    <row r="19" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+    </row>
+    <row r="20" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+    </row>
+    <row r="21" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+    </row>
+    <row r="23" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+    </row>
+    <row r="24" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+    </row>
+    <row r="25" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+    </row>
+    <row r="26" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+    </row>
+    <row r="27" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+    </row>
+    <row r="28" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+    </row>
+    <row r="29" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="3"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="55" orientation="landscape" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ajout de retours d'exp (REX)
</commit_message>
<xml_diff>
--- a/Docs/Retour d'expérience/Retour d'expérience.xlsx
+++ b/Docs/Retour d'expérience/Retour d'expérience.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Cours\Lowtech\WINS 2026\Four solaire\Docs\Retour d'expérience\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3ACB41D-EE0A-441C-A58A-672D047B11B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FA25AFB-6071-43D6-9835-22EAEA0FD0E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Problèmes_Solutions" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="77">
   <si>
     <t>Retour d'expérience sur la fabrication, le montage et l'utilisation  du four</t>
   </si>
@@ -215,7 +215,52 @@
     <t>Remarques</t>
   </si>
   <si>
-    <t>La barre symbolique des 100°C a été franchie</t>
+    <t>3/2</t>
+  </si>
+  <si>
+    <t>Déflecteur Bas</t>
+  </si>
+  <si>
+    <t>Le réglage de l'angle n'a pas l'air assez fin.</t>
+  </si>
+  <si>
+    <t>Vitre</t>
+  </si>
+  <si>
+    <t>Le pourtour de la vitre n'a pas l'air assez étanche, particulièrement vers le haut.</t>
+  </si>
+  <si>
+    <t>Plaque CP dessous-devant</t>
+  </si>
+  <si>
+    <t>Dessous</t>
+  </si>
+  <si>
+    <t>3 vis semble léger pour retenir la vitre</t>
+  </si>
+  <si>
+    <t>Ajouter deux vis supplémentaires. Changer la longueur des vis centrales pour du 30mm.</t>
+  </si>
+  <si>
+    <t>Changer le système qui maintient la vis en place.</t>
+  </si>
+  <si>
+    <t>La barre symbolique des 100°C a été franchie. Les parois n'ont pas été isolées avec le liège actuellement</t>
+  </si>
+  <si>
+    <t>Isolation</t>
+  </si>
+  <si>
+    <t>Les panneaux de liège en 20mm sont disponible qu'à un endroit vers Pompaple</t>
+  </si>
+  <si>
+    <t>Passer en deux épaisseurs de 10mm, disponible en magasin de bricolage</t>
+  </si>
+  <si>
+    <t>Changer l'isolant pour des panneaux en laine de mouton</t>
+  </si>
+  <si>
+    <t>Ajouter une meilleure isolation que le CP 6mm qui ferme. Un tasseau de 30x30x398mm est utilisé et calé dans le haut du four pour limiter les fuites par convection. Il faudrait aussi ajouter un joint silicone Haute-température tout autour de la vitre.</t>
   </si>
 </sst>
 </file>
@@ -308,7 +353,7 @@
     <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -594,7 +639,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" style="1" customWidth="1"/>
@@ -786,6 +831,68 @@
       </c>
       <c r="E12" s="1" t="s">
         <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -815,7 +922,7 @@
     <col min="8" max="8" width="33.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="35" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23.5703125" style="4" customWidth="1"/>
-    <col min="11" max="11" width="41" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="94.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="11.42578125" style="4"/>
   </cols>
   <sheetData>
@@ -873,8 +980,8 @@
       <c r="F2" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="G2" s="9">
-        <v>46253</v>
+      <c r="G2" s="9" t="s">
+        <v>61</v>
       </c>
       <c r="H2" s="3">
         <v>27.4</v>
@@ -886,7 +993,7 @@
         <v>59</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>